<commit_message>
Feat: UI_Option 일부 수정
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Localization/English.xlsx
+++ b/Assets/StreamingAssets/Localization/English.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Unity\AirNHook\Assets\StreamingAssets\Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29524789-1A11-4090-ACE5-2C9DD63BA8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA24053-DC96-4E2B-9380-0EED417F262A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4335" yWindow="1200" windowWidth="22785" windowHeight="13485" xr2:uid="{03AB7020-0D5B-4C42-B659-F913FE2E7807}"/>
+    <workbookView xWindow="4680" yWindow="1545" windowWidth="22785" windowHeight="13485" xr2:uid="{03AB7020-0D5B-4C42-B659-F913FE2E7807}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>id</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -155,6 +155,10 @@
   </si>
   <si>
     <t>Start Stage</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sorry, Current UserTestBuild does not contain SOUNDS yet!!!</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -595,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D177C49-BEC9-445E-96B9-01949D401546}">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="2" width="51.5" customWidth="1"/>
@@ -729,107 +733,115 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.25" thickBot="1">
+    <row r="17" spans="1:2" ht="28.5" thickBot="1">
       <c r="A17" s="1">
-        <v>2001</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>8</v>
+        <v>1015</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17.25" thickBot="1">
       <c r="A18" s="1">
-        <v>2002</v>
+        <v>2001</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17.25" thickBot="1">
       <c r="A19" s="1">
-        <v>2003</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>10</v>
+        <v>2002</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" thickBot="1">
       <c r="A20" s="1">
-        <v>2004</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>11</v>
+        <v>2003</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="17.25" thickBot="1">
       <c r="A21" s="1">
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="17.25" thickBot="1">
       <c r="A22" s="1">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17.25" thickBot="1">
       <c r="A23" s="1">
-        <v>2007</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>5</v>
+        <v>2006</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="17.25" thickBot="1">
       <c r="A24" s="1">
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="17.25" thickBot="1">
       <c r="A25" s="1">
-        <v>2009</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>7</v>
+        <v>2008</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="17.25" thickBot="1">
       <c r="A26" s="1">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="17.25" thickBot="1">
       <c r="A27" s="1">
-        <v>2101</v>
+        <v>2010</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="17.25" thickBot="1">
       <c r="A28" s="1">
-        <v>4001</v>
+        <v>2101</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="17.25" thickBot="1">
       <c r="A29" s="1">
+        <v>4001</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="17.25" thickBot="1">
+      <c r="A30" s="1">
         <v>4002</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B30" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>